<commit_message>
feat: expand audit workflows and mobile auditor experience
</commit_message>
<xml_diff>
--- a/src/Web/public/templates/AMS_Asset_Import_Template.xlsx
+++ b/src/Web/public/templates/AMS_Asset_Import_Template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset Import" sheetId="1" r:id="Re4057642b60049a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R64d2001e794d42bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset Import" sheetId="1" r:id="R7f0a706ff6dd452e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R3f411e3915f24272"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -196,7 +196,7 @@
         <x:color rgb="FFA60010"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCEBED"/>
         </x:patternFill>
       </x:fill>
@@ -666,23 +666,15 @@
         <x:v>WarrantyPeriodEndDate</x:v>
       </x:c>
       <x:c r="BM1" s="5" t="str">
-        <x:v>Auditor Name</x:v>
+        <x:v>Make</x:v>
       </x:c>
       <x:c r="BN1" s="5" t="str">
-        <x:v>Auditor Company Name</x:v>
-      </x:c>
-      <x:c r="BO1" s="5" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="BP1" s="5" t="str">
-        <x:v>Auditor Remarks</x:v>
-      </x:c>
-      <x:c r="BQ1" s="5" t="str">
-        <x:v>Make</x:v>
-      </x:c>
-      <x:c r="BR1" s="5" t="str">
         <x:v>Model</x:v>
       </x:c>
+      <x:c r="BO1"/>
+      <x:c r="BP1"/>
+      <x:c r="BQ1"/>
+      <x:c r="BR1"/>
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
       <x:c r="A2" s="8"/>
@@ -2238,7 +2230,7 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="12" t="str">
-        <x:v>Column dictionary (70 standard columns)</x:v>
+        <x:v>Column dictionary (66 standard columns)</x:v>
       </x:c>
       <x:c r="B11" s="12"/>
       <x:c r="C11" s="12"/>
@@ -3351,11 +3343,11 @@
       </x:c>
     </x:row>
     <x:row r="77">
-      <x:c r="A77" s="27" t="n">
+      <x:c r="A77" s="27" t="str">
         <x:v>65</x:v>
       </x:c>
       <x:c r="B77" s="21" t="str">
-        <x:v>Auditor Name</x:v>
+        <x:v>Make</x:v>
       </x:c>
       <x:c r="C77" s="21" t="str">
         <x:v>No</x:v>
@@ -3364,15 +3356,15 @@
         <x:v>Text</x:v>
       </x:c>
       <x:c r="E77" s="21" t="str">
-        <x:v>Enter the asset's auditor name value when available; otherwise leave blank.</x:v>
+        <x:v>Enter the asset's make value when available; otherwise leave blank.</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
-      <x:c r="A78" s="27" t="n">
+      <x:c r="A78" s="27" t="str">
         <x:v>66</x:v>
       </x:c>
       <x:c r="B78" s="21" t="str">
-        <x:v>Auditor Company Name</x:v>
+        <x:v>Model</x:v>
       </x:c>
       <x:c r="C78" s="21" t="str">
         <x:v>No</x:v>
@@ -3381,76 +3373,36 @@
         <x:v>Text</x:v>
       </x:c>
       <x:c r="E78" s="21" t="str">
-        <x:v>Enter the asset's auditor company name value when available; otherwise leave blank.</x:v>
+        <x:v>Enter the asset's model value when available; otherwise leave blank.</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
-      <x:c r="A79" s="27" t="n">
-        <x:v>67</x:v>
-      </x:c>
-      <x:c r="B79" s="21" t="str">
-        <x:v>Verified</x:v>
-      </x:c>
-      <x:c r="C79" s="21" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="D79" s="21" t="str">
-        <x:v>Text</x:v>
-      </x:c>
-      <x:c r="E79" s="21" t="str">
-        <x:v>Audit verification result, for example Yes, No, Verified or Pending.</x:v>
-      </x:c>
+      <x:c r="A79"/>
+      <x:c r="B79"/>
+      <x:c r="C79"/>
+      <x:c r="D79"/>
+      <x:c r="E79"/>
     </x:row>
     <x:row r="80">
-      <x:c r="A80" s="27" t="n">
-        <x:v>68</x:v>
-      </x:c>
-      <x:c r="B80" s="21" t="str">
-        <x:v>Auditor Remarks</x:v>
-      </x:c>
-      <x:c r="C80" s="21" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="D80" s="21" t="str">
-        <x:v>Text</x:v>
-      </x:c>
-      <x:c r="E80" s="21" t="str">
-        <x:v>Enter the asset's auditor remarks value when available; otherwise leave blank.</x:v>
-      </x:c>
+      <x:c r="A80"/>
+      <x:c r="B80"/>
+      <x:c r="C80"/>
+      <x:c r="D80"/>
+      <x:c r="E80"/>
     </x:row>
     <x:row r="81">
-      <x:c r="A81" s="27" t="n">
-        <x:v>69</x:v>
-      </x:c>
-      <x:c r="B81" s="21" t="str">
-        <x:v>Make</x:v>
-      </x:c>
-      <x:c r="C81" s="21" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="D81" s="21" t="str">
-        <x:v>Text</x:v>
-      </x:c>
-      <x:c r="E81" s="21" t="str">
-        <x:v>Enter the asset's make value when available; otherwise leave blank.</x:v>
-      </x:c>
+      <x:c r="A81"/>
+      <x:c r="B81"/>
+      <x:c r="C81"/>
+      <x:c r="D81"/>
+      <x:c r="E81"/>
     </x:row>
     <x:row r="82">
-      <x:c r="A82" s="27" t="n">
-        <x:v>70</x:v>
-      </x:c>
-      <x:c r="B82" s="21" t="str">
-        <x:v>Model</x:v>
-      </x:c>
-      <x:c r="C82" s="21" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="D82" s="21" t="str">
-        <x:v>Text</x:v>
-      </x:c>
-      <x:c r="E82" s="21" t="str">
-        <x:v>Enter the asset's model value when available; otherwise leave blank.</x:v>
-      </x:c>
+      <x:c r="A82"/>
+      <x:c r="B82"/>
+      <x:c r="C82"/>
+      <x:c r="D82"/>
+      <x:c r="E82"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>